<commit_message>
modifica colonne su file excel
</commit_message>
<xml_diff>
--- a/Lezione 1 - Iris_Lab_Excel.xlsx
+++ b/Lezione 1 - Iris_Lab_Excel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gmorelli\IdeaProjects\B3099---LABORATORIO-DI-OTTIMIZZAZIONE-INTELLIGENZA-ARTIFICIALE-E-MACHINE-LEARNING---2025-2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24CAD2D0-D190-4F57-A666-CFDA9C061E36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53270896-6B7C-4F72-A55B-92FE16D0F8BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Istruzioni" sheetId="1" r:id="rId1"/>
@@ -20,9 +20,8 @@
     <sheet name="Scatter" sheetId="6" r:id="rId5"/>
     <sheet name="Preprocessing" sheetId="4" r:id="rId6"/>
     <sheet name="Outlier_IQR" sheetId="5" r:id="rId7"/>
-    <sheet name="Dettagli1" sheetId="12" r:id="rId8"/>
-    <sheet name="Chi Quadro" sheetId="11" r:id="rId9"/>
-    <sheet name="Consegna" sheetId="8" r:id="rId10"/>
+    <sheet name="Chi Quadro" sheetId="11" r:id="rId8"/>
+    <sheet name="Consegna" sheetId="8" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Dati_grezzi!$A$1:$E$151</definedName>
@@ -30,7 +29,7 @@
   </definedNames>
   <calcPr calcId="191028"/>
   <pivotCaches>
-    <pivotCache cacheId="5" r:id="rId11"/>
+    <pivotCache cacheId="0" r:id="rId10"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -52,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="76">
   <si>
     <t>Laboratorio 1 – Iris (Excel 365, IT)</t>
   </si>
@@ -282,9 +281,6 @@
   <si>
     <t>Test T</t>
   </si>
-  <si>
-    <t>Dettagli per Somma di Contatore - species: virginica, bin: Alto</t>
-  </si>
 </sst>
 </file>
 
@@ -353,7 +349,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -377,7 +373,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -1183,7 +1178,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{30BC0138-36EC-407B-9CFD-362C426E4BE0}" name="Tabella pivot2" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valori" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{30BC0138-36EC-407B-9CFD-362C426E4BE0}" name="Tabella pivot2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valori" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:E8" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="3">
     <pivotField axis="axisRow" showAll="0">
@@ -1251,18 +1246,6 @@
     </ext>
   </extLst>
 </pivotTableDefinition>
-</file>
-
-<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{54BDAE5D-A46C-4D6C-AC97-7707B981486E}" name="Tabella1" displayName="Tabella1" ref="A3:C50" totalsRowShown="0">
-  <autoFilter ref="A3:C50" xr:uid="{54BDAE5D-A46C-4D6C-AC97-7707B981486E}"/>
-  <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{833068E0-2309-4183-98A7-7FBCA329A4D3}" name="species"/>
-    <tableColumn id="2" xr3:uid="{8B1BE7E6-6C4E-46F7-966C-58C1023B6EEA}" name="bin"/>
-    <tableColumn id="3" xr3:uid="{AD18D3FE-4A6B-4168-BA91-4CB7D5B4CBC2}" name="Contatore"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1606,57 +1589,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:A9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="120" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:1" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
-        <v>69</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:O151"/>
+  <dimension ref="A1:J151"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19" customWidth="1"/>
@@ -1668,11 +1603,10 @@
     <col min="7" max="7" width="12.28515625" customWidth="1"/>
     <col min="8" max="8" width="10.5703125" customWidth="1"/>
     <col min="9" max="9" width="12" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="1.85546875" customWidth="1"/>
-    <col min="15" max="15" width="23" customWidth="1"/>
+    <col min="10" max="10" width="23" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>9</v>
       </c>
@@ -1697,11 +1631,11 @@
       <c r="I1" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="O1" t="s">
+      <c r="J1" s="10" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>5.0999999999999996</v>
       </c>
@@ -1718,7 +1652,7 @@
         <v>17</v>
       </c>
       <c r="F2" t="str">
-        <f>IF(Dati_grezzi!C2&lt;=$O$2,"Basso",IF(C2&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C2&lt;=$J$2,"Basso",IF(C2&lt;=$J$3,"Medio","Alto"))</f>
         <v>Basso</v>
       </c>
       <c r="G2">
@@ -1728,12 +1662,12 @@
         <f>TTEST(C2:C51,C52:C101,2,3)</f>
         <v>9.9344329575875926E-46</v>
       </c>
-      <c r="O2">
+      <c r="J2">
         <f>_xlfn.PERCENTILE.INC(Dati_grezzi!C2:C151,0.3333)</f>
         <v>2.6278699999999957</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>4.9000000000000004</v>
       </c>
@@ -1750,18 +1684,18 @@
         <v>17</v>
       </c>
       <c r="F3" t="str">
-        <f>IF(Dati_grezzi!C3&lt;=$O$2,"Basso",IF(C3&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C3&lt;=$J$2,"Basso",IF(C3&lt;=$J$3,"Medio","Alto"))</f>
         <v>Basso</v>
       </c>
       <c r="G3">
         <v>1</v>
       </c>
-      <c r="O3">
+      <c r="J3">
         <f>_xlfn.PERCENTILE.INC(Dati_grezzi!C2:C151,0.66666)</f>
         <v>4.9000000000000004</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>4.7</v>
       </c>
@@ -1778,14 +1712,14 @@
         <v>17</v>
       </c>
       <c r="F4" t="str">
-        <f>IF(Dati_grezzi!C4&lt;=$O$2,"Basso",IF(C4&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C4&lt;=$J$2,"Basso",IF(C4&lt;=$J$3,"Medio","Alto"))</f>
         <v>Basso</v>
       </c>
       <c r="G4">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4.5999999999999996</v>
       </c>
@@ -1802,14 +1736,14 @@
         <v>17</v>
       </c>
       <c r="F5" t="str">
-        <f>IF(Dati_grezzi!C5&lt;=$O$2,"Basso",IF(C5&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C5&lt;=$J$2,"Basso",IF(C5&lt;=$J$3,"Medio","Alto"))</f>
         <v>Basso</v>
       </c>
       <c r="G5">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1826,14 +1760,14 @@
         <v>17</v>
       </c>
       <c r="F6" t="str">
-        <f>IF(Dati_grezzi!C6&lt;=$O$2,"Basso",IF(C6&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C6&lt;=$J$2,"Basso",IF(C6&lt;=$J$3,"Medio","Alto"))</f>
         <v>Basso</v>
       </c>
       <c r="G6">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>5.4</v>
       </c>
@@ -1850,14 +1784,14 @@
         <v>17</v>
       </c>
       <c r="F7" t="str">
-        <f>IF(Dati_grezzi!C7&lt;=$O$2,"Basso",IF(C7&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C7&lt;=$J$2,"Basso",IF(C7&lt;=$J$3,"Medio","Alto"))</f>
         <v>Basso</v>
       </c>
       <c r="G7">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>4.5999999999999996</v>
       </c>
@@ -1874,14 +1808,14 @@
         <v>17</v>
       </c>
       <c r="F8" t="str">
-        <f>IF(Dati_grezzi!C8&lt;=$O$2,"Basso",IF(C8&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C8&lt;=$J$2,"Basso",IF(C8&lt;=$J$3,"Medio","Alto"))</f>
         <v>Basso</v>
       </c>
       <c r="G8">
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>5</v>
       </c>
@@ -1898,14 +1832,14 @@
         <v>17</v>
       </c>
       <c r="F9" t="str">
-        <f>IF(Dati_grezzi!C9&lt;=$O$2,"Basso",IF(C9&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C9&lt;=$J$2,"Basso",IF(C9&lt;=$J$3,"Medio","Alto"))</f>
         <v>Basso</v>
       </c>
       <c r="G9">
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>4.4000000000000004</v>
       </c>
@@ -1922,14 +1856,14 @@
         <v>17</v>
       </c>
       <c r="F10" t="str">
-        <f>IF(Dati_grezzi!C10&lt;=$O$2,"Basso",IF(C10&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C10&lt;=$J$2,"Basso",IF(C10&lt;=$J$3,"Medio","Alto"))</f>
         <v>Basso</v>
       </c>
       <c r="G10">
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>4.9000000000000004</v>
       </c>
@@ -1946,14 +1880,14 @@
         <v>17</v>
       </c>
       <c r="F11" t="str">
-        <f>IF(Dati_grezzi!C11&lt;=$O$2,"Basso",IF(C11&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C11&lt;=$J$2,"Basso",IF(C11&lt;=$J$3,"Medio","Alto"))</f>
         <v>Basso</v>
       </c>
       <c r="G11">
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>5.4</v>
       </c>
@@ -1970,14 +1904,14 @@
         <v>17</v>
       </c>
       <c r="F12" t="str">
-        <f>IF(Dati_grezzi!C12&lt;=$O$2,"Basso",IF(C12&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C12&lt;=$J$2,"Basso",IF(C12&lt;=$J$3,"Medio","Alto"))</f>
         <v>Basso</v>
       </c>
       <c r="G12">
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>4.8</v>
       </c>
@@ -1994,14 +1928,14 @@
         <v>17</v>
       </c>
       <c r="F13" t="str">
-        <f>IF(Dati_grezzi!C13&lt;=$O$2,"Basso",IF(C13&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C13&lt;=$J$2,"Basso",IF(C13&lt;=$J$3,"Medio","Alto"))</f>
         <v>Basso</v>
       </c>
       <c r="G13">
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>4.8</v>
       </c>
@@ -2018,14 +1952,14 @@
         <v>17</v>
       </c>
       <c r="F14" t="str">
-        <f>IF(Dati_grezzi!C14&lt;=$O$2,"Basso",IF(C14&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C14&lt;=$J$2,"Basso",IF(C14&lt;=$J$3,"Medio","Alto"))</f>
         <v>Basso</v>
       </c>
       <c r="G14">
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>4.3</v>
       </c>
@@ -2042,14 +1976,14 @@
         <v>17</v>
       </c>
       <c r="F15" t="str">
-        <f>IF(Dati_grezzi!C15&lt;=$O$2,"Basso",IF(C15&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C15&lt;=$J$2,"Basso",IF(C15&lt;=$J$3,"Medio","Alto"))</f>
         <v>Basso</v>
       </c>
       <c r="G15">
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>5.8</v>
       </c>
@@ -2066,7 +2000,7 @@
         <v>17</v>
       </c>
       <c r="F16" t="str">
-        <f>IF(Dati_grezzi!C16&lt;=$O$2,"Basso",IF(C16&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C16&lt;=$J$2,"Basso",IF(C16&lt;=$J$3,"Medio","Alto"))</f>
         <v>Basso</v>
       </c>
       <c r="G16">
@@ -2090,7 +2024,7 @@
         <v>17</v>
       </c>
       <c r="F17" t="str">
-        <f>IF(Dati_grezzi!C17&lt;=$O$2,"Basso",IF(C17&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C17&lt;=$J$2,"Basso",IF(C17&lt;=$J$3,"Medio","Alto"))</f>
         <v>Basso</v>
       </c>
       <c r="G17">
@@ -2114,7 +2048,7 @@
         <v>17</v>
       </c>
       <c r="F18" t="str">
-        <f>IF(Dati_grezzi!C18&lt;=$O$2,"Basso",IF(C18&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C18&lt;=$J$2,"Basso",IF(C18&lt;=$J$3,"Medio","Alto"))</f>
         <v>Basso</v>
       </c>
       <c r="G18">
@@ -2138,7 +2072,7 @@
         <v>17</v>
       </c>
       <c r="F19" t="str">
-        <f>IF(Dati_grezzi!C19&lt;=$O$2,"Basso",IF(C19&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C19&lt;=$J$2,"Basso",IF(C19&lt;=$J$3,"Medio","Alto"))</f>
         <v>Basso</v>
       </c>
       <c r="G19">
@@ -2162,7 +2096,7 @@
         <v>17</v>
       </c>
       <c r="F20" t="str">
-        <f>IF(Dati_grezzi!C20&lt;=$O$2,"Basso",IF(C20&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C20&lt;=$J$2,"Basso",IF(C20&lt;=$J$3,"Medio","Alto"))</f>
         <v>Basso</v>
       </c>
       <c r="G20">
@@ -2186,7 +2120,7 @@
         <v>17</v>
       </c>
       <c r="F21" t="str">
-        <f>IF(Dati_grezzi!C21&lt;=$O$2,"Basso",IF(C21&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C21&lt;=$J$2,"Basso",IF(C21&lt;=$J$3,"Medio","Alto"))</f>
         <v>Basso</v>
       </c>
       <c r="G21">
@@ -2210,7 +2144,7 @@
         <v>17</v>
       </c>
       <c r="F22" t="str">
-        <f>IF(Dati_grezzi!C22&lt;=$O$2,"Basso",IF(C22&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C22&lt;=$J$2,"Basso",IF(C22&lt;=$J$3,"Medio","Alto"))</f>
         <v>Basso</v>
       </c>
       <c r="G22">
@@ -2234,7 +2168,7 @@
         <v>17</v>
       </c>
       <c r="F23" t="str">
-        <f>IF(Dati_grezzi!C23&lt;=$O$2,"Basso",IF(C23&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C23&lt;=$J$2,"Basso",IF(C23&lt;=$J$3,"Medio","Alto"))</f>
         <v>Basso</v>
       </c>
       <c r="G23">
@@ -2258,7 +2192,7 @@
         <v>17</v>
       </c>
       <c r="F24" t="str">
-        <f>IF(Dati_grezzi!C24&lt;=$O$2,"Basso",IF(C24&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C24&lt;=$J$2,"Basso",IF(C24&lt;=$J$3,"Medio","Alto"))</f>
         <v>Basso</v>
       </c>
       <c r="G24">
@@ -2282,7 +2216,7 @@
         <v>17</v>
       </c>
       <c r="F25" t="str">
-        <f>IF(Dati_grezzi!C25&lt;=$O$2,"Basso",IF(C25&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C25&lt;=$J$2,"Basso",IF(C25&lt;=$J$3,"Medio","Alto"))</f>
         <v>Basso</v>
       </c>
       <c r="G25">
@@ -2306,7 +2240,7 @@
         <v>17</v>
       </c>
       <c r="F26" t="str">
-        <f>IF(Dati_grezzi!C26&lt;=$O$2,"Basso",IF(C26&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C26&lt;=$J$2,"Basso",IF(C26&lt;=$J$3,"Medio","Alto"))</f>
         <v>Basso</v>
       </c>
       <c r="G26">
@@ -2330,7 +2264,7 @@
         <v>17</v>
       </c>
       <c r="F27" t="str">
-        <f>IF(Dati_grezzi!C27&lt;=$O$2,"Basso",IF(C27&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C27&lt;=$J$2,"Basso",IF(C27&lt;=$J$3,"Medio","Alto"))</f>
         <v>Basso</v>
       </c>
       <c r="G27">
@@ -2354,7 +2288,7 @@
         <v>17</v>
       </c>
       <c r="F28" t="str">
-        <f>IF(Dati_grezzi!C28&lt;=$O$2,"Basso",IF(C28&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C28&lt;=$J$2,"Basso",IF(C28&lt;=$J$3,"Medio","Alto"))</f>
         <v>Basso</v>
       </c>
       <c r="G28">
@@ -2378,7 +2312,7 @@
         <v>17</v>
       </c>
       <c r="F29" t="str">
-        <f>IF(Dati_grezzi!C29&lt;=$O$2,"Basso",IF(C29&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C29&lt;=$J$2,"Basso",IF(C29&lt;=$J$3,"Medio","Alto"))</f>
         <v>Basso</v>
       </c>
       <c r="G29">
@@ -2402,7 +2336,7 @@
         <v>17</v>
       </c>
       <c r="F30" t="str">
-        <f>IF(Dati_grezzi!C30&lt;=$O$2,"Basso",IF(C30&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C30&lt;=$J$2,"Basso",IF(C30&lt;=$J$3,"Medio","Alto"))</f>
         <v>Basso</v>
       </c>
       <c r="G30">
@@ -2426,7 +2360,7 @@
         <v>17</v>
       </c>
       <c r="F31" t="str">
-        <f>IF(Dati_grezzi!C31&lt;=$O$2,"Basso",IF(C31&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C31&lt;=$J$2,"Basso",IF(C31&lt;=$J$3,"Medio","Alto"))</f>
         <v>Basso</v>
       </c>
       <c r="G31">
@@ -2450,7 +2384,7 @@
         <v>17</v>
       </c>
       <c r="F32" t="str">
-        <f>IF(Dati_grezzi!C32&lt;=$O$2,"Basso",IF(C32&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C32&lt;=$J$2,"Basso",IF(C32&lt;=$J$3,"Medio","Alto"))</f>
         <v>Basso</v>
       </c>
       <c r="G32">
@@ -2474,7 +2408,7 @@
         <v>17</v>
       </c>
       <c r="F33" t="str">
-        <f>IF(Dati_grezzi!C33&lt;=$O$2,"Basso",IF(C33&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C33&lt;=$J$2,"Basso",IF(C33&lt;=$J$3,"Medio","Alto"))</f>
         <v>Basso</v>
       </c>
       <c r="G33">
@@ -2498,7 +2432,7 @@
         <v>17</v>
       </c>
       <c r="F34" t="str">
-        <f>IF(Dati_grezzi!C34&lt;=$O$2,"Basso",IF(C34&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C34&lt;=$J$2,"Basso",IF(C34&lt;=$J$3,"Medio","Alto"))</f>
         <v>Basso</v>
       </c>
       <c r="G34">
@@ -2522,7 +2456,7 @@
         <v>17</v>
       </c>
       <c r="F35" t="str">
-        <f>IF(Dati_grezzi!C35&lt;=$O$2,"Basso",IF(C35&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C35&lt;=$J$2,"Basso",IF(C35&lt;=$J$3,"Medio","Alto"))</f>
         <v>Basso</v>
       </c>
       <c r="G35">
@@ -2546,7 +2480,7 @@
         <v>17</v>
       </c>
       <c r="F36" t="str">
-        <f>IF(Dati_grezzi!C36&lt;=$O$2,"Basso",IF(C36&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C36&lt;=$J$2,"Basso",IF(C36&lt;=$J$3,"Medio","Alto"))</f>
         <v>Basso</v>
       </c>
       <c r="G36">
@@ -2570,7 +2504,7 @@
         <v>17</v>
       </c>
       <c r="F37" t="str">
-        <f>IF(Dati_grezzi!C37&lt;=$O$2,"Basso",IF(C37&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C37&lt;=$J$2,"Basso",IF(C37&lt;=$J$3,"Medio","Alto"))</f>
         <v>Basso</v>
       </c>
       <c r="G37">
@@ -2594,7 +2528,7 @@
         <v>17</v>
       </c>
       <c r="F38" t="str">
-        <f>IF(Dati_grezzi!C38&lt;=$O$2,"Basso",IF(C38&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C38&lt;=$J$2,"Basso",IF(C38&lt;=$J$3,"Medio","Alto"))</f>
         <v>Basso</v>
       </c>
       <c r="G38">
@@ -2618,7 +2552,7 @@
         <v>17</v>
       </c>
       <c r="F39" t="str">
-        <f>IF(Dati_grezzi!C39&lt;=$O$2,"Basso",IF(C39&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C39&lt;=$J$2,"Basso",IF(C39&lt;=$J$3,"Medio","Alto"))</f>
         <v>Basso</v>
       </c>
       <c r="G39">
@@ -2642,7 +2576,7 @@
         <v>17</v>
       </c>
       <c r="F40" t="str">
-        <f>IF(Dati_grezzi!C40&lt;=$O$2,"Basso",IF(C40&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C40&lt;=$J$2,"Basso",IF(C40&lt;=$J$3,"Medio","Alto"))</f>
         <v>Basso</v>
       </c>
       <c r="G40">
@@ -2666,7 +2600,7 @@
         <v>17</v>
       </c>
       <c r="F41" t="str">
-        <f>IF(Dati_grezzi!C41&lt;=$O$2,"Basso",IF(C41&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C41&lt;=$J$2,"Basso",IF(C41&lt;=$J$3,"Medio","Alto"))</f>
         <v>Basso</v>
       </c>
       <c r="G41">
@@ -2690,7 +2624,7 @@
         <v>17</v>
       </c>
       <c r="F42" t="str">
-        <f>IF(Dati_grezzi!C42&lt;=$O$2,"Basso",IF(C42&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C42&lt;=$J$2,"Basso",IF(C42&lt;=$J$3,"Medio","Alto"))</f>
         <v>Basso</v>
       </c>
       <c r="G42">
@@ -2714,7 +2648,7 @@
         <v>17</v>
       </c>
       <c r="F43" t="str">
-        <f>IF(Dati_grezzi!C43&lt;=$O$2,"Basso",IF(C43&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C43&lt;=$J$2,"Basso",IF(C43&lt;=$J$3,"Medio","Alto"))</f>
         <v>Basso</v>
       </c>
       <c r="G43">
@@ -2738,7 +2672,7 @@
         <v>17</v>
       </c>
       <c r="F44" t="str">
-        <f>IF(Dati_grezzi!C44&lt;=$O$2,"Basso",IF(C44&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C44&lt;=$J$2,"Basso",IF(C44&lt;=$J$3,"Medio","Alto"))</f>
         <v>Basso</v>
       </c>
       <c r="G44">
@@ -2762,7 +2696,7 @@
         <v>17</v>
       </c>
       <c r="F45" t="str">
-        <f>IF(Dati_grezzi!C45&lt;=$O$2,"Basso",IF(C45&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C45&lt;=$J$2,"Basso",IF(C45&lt;=$J$3,"Medio","Alto"))</f>
         <v>Basso</v>
       </c>
       <c r="G45">
@@ -2786,7 +2720,7 @@
         <v>17</v>
       </c>
       <c r="F46" t="str">
-        <f>IF(Dati_grezzi!C46&lt;=$O$2,"Basso",IF(C46&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C46&lt;=$J$2,"Basso",IF(C46&lt;=$J$3,"Medio","Alto"))</f>
         <v>Basso</v>
       </c>
       <c r="G46">
@@ -2810,7 +2744,7 @@
         <v>17</v>
       </c>
       <c r="F47" t="str">
-        <f>IF(Dati_grezzi!C47&lt;=$O$2,"Basso",IF(C47&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C47&lt;=$J$2,"Basso",IF(C47&lt;=$J$3,"Medio","Alto"))</f>
         <v>Basso</v>
       </c>
       <c r="G47">
@@ -2834,7 +2768,7 @@
         <v>17</v>
       </c>
       <c r="F48" t="str">
-        <f>IF(Dati_grezzi!C48&lt;=$O$2,"Basso",IF(C48&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C48&lt;=$J$2,"Basso",IF(C48&lt;=$J$3,"Medio","Alto"))</f>
         <v>Basso</v>
       </c>
       <c r="G48">
@@ -2858,7 +2792,7 @@
         <v>17</v>
       </c>
       <c r="F49" t="str">
-        <f>IF(Dati_grezzi!C49&lt;=$O$2,"Basso",IF(C49&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C49&lt;=$J$2,"Basso",IF(C49&lt;=$J$3,"Medio","Alto"))</f>
         <v>Basso</v>
       </c>
       <c r="G49">
@@ -2882,7 +2816,7 @@
         <v>17</v>
       </c>
       <c r="F50" t="str">
-        <f>IF(Dati_grezzi!C50&lt;=$O$2,"Basso",IF(C50&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C50&lt;=$J$2,"Basso",IF(C50&lt;=$J$3,"Medio","Alto"))</f>
         <v>Basso</v>
       </c>
       <c r="G50">
@@ -2906,7 +2840,7 @@
         <v>17</v>
       </c>
       <c r="F51" t="str">
-        <f>IF(Dati_grezzi!C51&lt;=$O$2,"Basso",IF(C51&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C51&lt;=$J$2,"Basso",IF(C51&lt;=$J$3,"Medio","Alto"))</f>
         <v>Basso</v>
       </c>
       <c r="G51">
@@ -2930,7 +2864,7 @@
         <v>18</v>
       </c>
       <c r="F52" t="str">
-        <f>IF(Dati_grezzi!C52&lt;=$O$2,"Basso",IF(C52&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C52&lt;=$J$2,"Basso",IF(C52&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G52">
@@ -2954,7 +2888,7 @@
         <v>18</v>
       </c>
       <c r="F53" t="str">
-        <f>IF(Dati_grezzi!C53&lt;=$O$2,"Basso",IF(C53&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C53&lt;=$J$2,"Basso",IF(C53&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G53">
@@ -2978,7 +2912,7 @@
         <v>18</v>
       </c>
       <c r="F54" t="str">
-        <f>IF(Dati_grezzi!C54&lt;=$O$2,"Basso",IF(C54&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C54&lt;=$J$2,"Basso",IF(C54&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G54">
@@ -3002,7 +2936,7 @@
         <v>18</v>
       </c>
       <c r="F55" t="str">
-        <f>IF(Dati_grezzi!C55&lt;=$O$2,"Basso",IF(C55&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C55&lt;=$J$2,"Basso",IF(C55&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G55">
@@ -3026,7 +2960,7 @@
         <v>18</v>
       </c>
       <c r="F56" t="str">
-        <f>IF(Dati_grezzi!C56&lt;=$O$2,"Basso",IF(C56&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C56&lt;=$J$2,"Basso",IF(C56&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G56">
@@ -3050,7 +2984,7 @@
         <v>18</v>
       </c>
       <c r="F57" t="str">
-        <f>IF(Dati_grezzi!C57&lt;=$O$2,"Basso",IF(C57&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C57&lt;=$J$2,"Basso",IF(C57&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G57">
@@ -3074,7 +3008,7 @@
         <v>18</v>
       </c>
       <c r="F58" t="str">
-        <f>IF(Dati_grezzi!C58&lt;=$O$2,"Basso",IF(C58&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C58&lt;=$J$2,"Basso",IF(C58&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G58">
@@ -3098,7 +3032,7 @@
         <v>18</v>
       </c>
       <c r="F59" t="str">
-        <f>IF(Dati_grezzi!C59&lt;=$O$2,"Basso",IF(C59&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C59&lt;=$J$2,"Basso",IF(C59&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G59">
@@ -3122,7 +3056,7 @@
         <v>18</v>
       </c>
       <c r="F60" t="str">
-        <f>IF(Dati_grezzi!C60&lt;=$O$2,"Basso",IF(C60&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C60&lt;=$J$2,"Basso",IF(C60&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G60">
@@ -3146,7 +3080,7 @@
         <v>18</v>
       </c>
       <c r="F61" t="str">
-        <f>IF(Dati_grezzi!C61&lt;=$O$2,"Basso",IF(C61&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C61&lt;=$J$2,"Basso",IF(C61&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G61">
@@ -3170,7 +3104,7 @@
         <v>18</v>
       </c>
       <c r="F62" t="str">
-        <f>IF(Dati_grezzi!C62&lt;=$O$2,"Basso",IF(C62&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C62&lt;=$J$2,"Basso",IF(C62&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G62">
@@ -3194,7 +3128,7 @@
         <v>18</v>
       </c>
       <c r="F63" t="str">
-        <f>IF(Dati_grezzi!C63&lt;=$O$2,"Basso",IF(C63&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C63&lt;=$J$2,"Basso",IF(C63&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G63">
@@ -3218,7 +3152,7 @@
         <v>18</v>
       </c>
       <c r="F64" t="str">
-        <f>IF(Dati_grezzi!C64&lt;=$O$2,"Basso",IF(C64&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C64&lt;=$J$2,"Basso",IF(C64&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G64">
@@ -3242,7 +3176,7 @@
         <v>18</v>
       </c>
       <c r="F65" t="str">
-        <f>IF(Dati_grezzi!C65&lt;=$O$2,"Basso",IF(C65&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C65&lt;=$J$2,"Basso",IF(C65&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G65">
@@ -3266,7 +3200,7 @@
         <v>18</v>
       </c>
       <c r="F66" t="str">
-        <f>IF(Dati_grezzi!C66&lt;=$O$2,"Basso",IF(C66&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C66&lt;=$J$2,"Basso",IF(C66&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G66">
@@ -3290,7 +3224,7 @@
         <v>18</v>
       </c>
       <c r="F67" t="str">
-        <f>IF(Dati_grezzi!C67&lt;=$O$2,"Basso",IF(C67&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C67&lt;=$J$2,"Basso",IF(C67&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G67">
@@ -3314,7 +3248,7 @@
         <v>18</v>
       </c>
       <c r="F68" t="str">
-        <f>IF(Dati_grezzi!C68&lt;=$O$2,"Basso",IF(C68&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C68&lt;=$J$2,"Basso",IF(C68&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G68">
@@ -3338,7 +3272,7 @@
         <v>18</v>
       </c>
       <c r="F69" t="str">
-        <f>IF(Dati_grezzi!C69&lt;=$O$2,"Basso",IF(C69&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C69&lt;=$J$2,"Basso",IF(C69&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G69">
@@ -3362,7 +3296,7 @@
         <v>18</v>
       </c>
       <c r="F70" t="str">
-        <f>IF(Dati_grezzi!C70&lt;=$O$2,"Basso",IF(C70&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C70&lt;=$J$2,"Basso",IF(C70&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G70">
@@ -3386,7 +3320,7 @@
         <v>18</v>
       </c>
       <c r="F71" t="str">
-        <f>IF(Dati_grezzi!C71&lt;=$O$2,"Basso",IF(C71&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C71&lt;=$J$2,"Basso",IF(C71&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G71">
@@ -3410,7 +3344,7 @@
         <v>18</v>
       </c>
       <c r="F72" t="str">
-        <f>IF(Dati_grezzi!C72&lt;=$O$2,"Basso",IF(C72&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C72&lt;=$J$2,"Basso",IF(C72&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G72">
@@ -3434,7 +3368,7 @@
         <v>18</v>
       </c>
       <c r="F73" t="str">
-        <f>IF(Dati_grezzi!C73&lt;=$O$2,"Basso",IF(C73&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C73&lt;=$J$2,"Basso",IF(C73&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G73">
@@ -3458,7 +3392,7 @@
         <v>18</v>
       </c>
       <c r="F74" t="str">
-        <f>IF(Dati_grezzi!C74&lt;=$O$2,"Basso",IF(C74&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C74&lt;=$J$2,"Basso",IF(C74&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G74">
@@ -3482,7 +3416,7 @@
         <v>18</v>
       </c>
       <c r="F75" t="str">
-        <f>IF(Dati_grezzi!C75&lt;=$O$2,"Basso",IF(C75&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C75&lt;=$J$2,"Basso",IF(C75&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G75">
@@ -3506,7 +3440,7 @@
         <v>18</v>
       </c>
       <c r="F76" t="str">
-        <f>IF(Dati_grezzi!C76&lt;=$O$2,"Basso",IF(C76&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C76&lt;=$J$2,"Basso",IF(C76&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G76">
@@ -3530,7 +3464,7 @@
         <v>18</v>
       </c>
       <c r="F77" t="str">
-        <f>IF(Dati_grezzi!C77&lt;=$O$2,"Basso",IF(C77&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C77&lt;=$J$2,"Basso",IF(C77&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G77">
@@ -3554,7 +3488,7 @@
         <v>18</v>
       </c>
       <c r="F78" t="str">
-        <f>IF(Dati_grezzi!C78&lt;=$O$2,"Basso",IF(C78&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C78&lt;=$J$2,"Basso",IF(C78&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G78">
@@ -3578,7 +3512,7 @@
         <v>18</v>
       </c>
       <c r="F79" t="str">
-        <f>IF(Dati_grezzi!C79&lt;=$O$2,"Basso",IF(C79&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C79&lt;=$J$2,"Basso",IF(C79&lt;=$J$3,"Medio","Alto"))</f>
         <v>Alto</v>
       </c>
       <c r="G79">
@@ -3602,7 +3536,7 @@
         <v>18</v>
       </c>
       <c r="F80" t="str">
-        <f>IF(Dati_grezzi!C80&lt;=$O$2,"Basso",IF(C80&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C80&lt;=$J$2,"Basso",IF(C80&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G80">
@@ -3626,7 +3560,7 @@
         <v>18</v>
       </c>
       <c r="F81" t="str">
-        <f>IF(Dati_grezzi!C81&lt;=$O$2,"Basso",IF(C81&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C81&lt;=$J$2,"Basso",IF(C81&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G81">
@@ -3650,7 +3584,7 @@
         <v>18</v>
       </c>
       <c r="F82" t="str">
-        <f>IF(Dati_grezzi!C82&lt;=$O$2,"Basso",IF(C82&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C82&lt;=$J$2,"Basso",IF(C82&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G82">
@@ -3674,7 +3608,7 @@
         <v>18</v>
       </c>
       <c r="F83" t="str">
-        <f>IF(Dati_grezzi!C83&lt;=$O$2,"Basso",IF(C83&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C83&lt;=$J$2,"Basso",IF(C83&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G83">
@@ -3698,7 +3632,7 @@
         <v>18</v>
       </c>
       <c r="F84" t="str">
-        <f>IF(Dati_grezzi!C84&lt;=$O$2,"Basso",IF(C84&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C84&lt;=$J$2,"Basso",IF(C84&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G84">
@@ -3722,7 +3656,7 @@
         <v>18</v>
       </c>
       <c r="F85" t="str">
-        <f>IF(Dati_grezzi!C85&lt;=$O$2,"Basso",IF(C85&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C85&lt;=$J$2,"Basso",IF(C85&lt;=$J$3,"Medio","Alto"))</f>
         <v>Alto</v>
       </c>
       <c r="G85">
@@ -3746,7 +3680,7 @@
         <v>18</v>
       </c>
       <c r="F86" t="str">
-        <f>IF(Dati_grezzi!C86&lt;=$O$2,"Basso",IF(C86&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C86&lt;=$J$2,"Basso",IF(C86&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G86">
@@ -3770,7 +3704,7 @@
         <v>18</v>
       </c>
       <c r="F87" t="str">
-        <f>IF(Dati_grezzi!C87&lt;=$O$2,"Basso",IF(C87&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C87&lt;=$J$2,"Basso",IF(C87&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G87">
@@ -3794,7 +3728,7 @@
         <v>18</v>
       </c>
       <c r="F88" t="str">
-        <f>IF(Dati_grezzi!C88&lt;=$O$2,"Basso",IF(C88&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C88&lt;=$J$2,"Basso",IF(C88&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G88">
@@ -3818,7 +3752,7 @@
         <v>18</v>
       </c>
       <c r="F89" t="str">
-        <f>IF(Dati_grezzi!C89&lt;=$O$2,"Basso",IF(C89&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C89&lt;=$J$2,"Basso",IF(C89&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G89">
@@ -3842,7 +3776,7 @@
         <v>18</v>
       </c>
       <c r="F90" t="str">
-        <f>IF(Dati_grezzi!C90&lt;=$O$2,"Basso",IF(C90&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C90&lt;=$J$2,"Basso",IF(C90&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G90">
@@ -3866,7 +3800,7 @@
         <v>18</v>
       </c>
       <c r="F91" t="str">
-        <f>IF(Dati_grezzi!C91&lt;=$O$2,"Basso",IF(C91&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C91&lt;=$J$2,"Basso",IF(C91&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G91">
@@ -3890,7 +3824,7 @@
         <v>18</v>
       </c>
       <c r="F92" t="str">
-        <f>IF(Dati_grezzi!C92&lt;=$O$2,"Basso",IF(C92&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C92&lt;=$J$2,"Basso",IF(C92&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G92">
@@ -3914,7 +3848,7 @@
         <v>18</v>
       </c>
       <c r="F93" t="str">
-        <f>IF(Dati_grezzi!C93&lt;=$O$2,"Basso",IF(C93&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C93&lt;=$J$2,"Basso",IF(C93&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G93">
@@ -3938,7 +3872,7 @@
         <v>18</v>
       </c>
       <c r="F94" t="str">
-        <f>IF(Dati_grezzi!C94&lt;=$O$2,"Basso",IF(C94&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C94&lt;=$J$2,"Basso",IF(C94&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G94">
@@ -3962,7 +3896,7 @@
         <v>18</v>
       </c>
       <c r="F95" t="str">
-        <f>IF(Dati_grezzi!C95&lt;=$O$2,"Basso",IF(C95&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C95&lt;=$J$2,"Basso",IF(C95&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G95">
@@ -3986,7 +3920,7 @@
         <v>18</v>
       </c>
       <c r="F96" t="str">
-        <f>IF(Dati_grezzi!C96&lt;=$O$2,"Basso",IF(C96&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C96&lt;=$J$2,"Basso",IF(C96&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G96">
@@ -4010,7 +3944,7 @@
         <v>18</v>
       </c>
       <c r="F97" t="str">
-        <f>IF(Dati_grezzi!C97&lt;=$O$2,"Basso",IF(C97&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C97&lt;=$J$2,"Basso",IF(C97&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G97">
@@ -4034,7 +3968,7 @@
         <v>18</v>
       </c>
       <c r="F98" t="str">
-        <f>IF(Dati_grezzi!C98&lt;=$O$2,"Basso",IF(C98&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C98&lt;=$J$2,"Basso",IF(C98&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G98">
@@ -4058,7 +3992,7 @@
         <v>18</v>
       </c>
       <c r="F99" t="str">
-        <f>IF(Dati_grezzi!C99&lt;=$O$2,"Basso",IF(C99&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C99&lt;=$J$2,"Basso",IF(C99&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G99">
@@ -4082,7 +4016,7 @@
         <v>18</v>
       </c>
       <c r="F100" t="str">
-        <f>IF(Dati_grezzi!C100&lt;=$O$2,"Basso",IF(C100&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C100&lt;=$J$2,"Basso",IF(C100&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G100">
@@ -4106,7 +4040,7 @@
         <v>18</v>
       </c>
       <c r="F101" t="str">
-        <f>IF(Dati_grezzi!C101&lt;=$O$2,"Basso",IF(C101&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C101&lt;=$J$2,"Basso",IF(C101&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G101">
@@ -4130,7 +4064,7 @@
         <v>19</v>
       </c>
       <c r="F102" t="str">
-        <f>IF(Dati_grezzi!C102&lt;=$O$2,"Basso",IF(C102&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C102&lt;=$J$2,"Basso",IF(C102&lt;=$J$3,"Medio","Alto"))</f>
         <v>Alto</v>
       </c>
       <c r="G102">
@@ -4154,7 +4088,7 @@
         <v>19</v>
       </c>
       <c r="F103" t="str">
-        <f>IF(Dati_grezzi!C103&lt;=$O$2,"Basso",IF(C103&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C103&lt;=$J$2,"Basso",IF(C103&lt;=$J$3,"Medio","Alto"))</f>
         <v>Alto</v>
       </c>
       <c r="G103">
@@ -4178,7 +4112,7 @@
         <v>19</v>
       </c>
       <c r="F104" t="str">
-        <f>IF(Dati_grezzi!C104&lt;=$O$2,"Basso",IF(C104&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C104&lt;=$J$2,"Basso",IF(C104&lt;=$J$3,"Medio","Alto"))</f>
         <v>Alto</v>
       </c>
       <c r="G104">
@@ -4202,7 +4136,7 @@
         <v>19</v>
       </c>
       <c r="F105" t="str">
-        <f>IF(Dati_grezzi!C105&lt;=$O$2,"Basso",IF(C105&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C105&lt;=$J$2,"Basso",IF(C105&lt;=$J$3,"Medio","Alto"))</f>
         <v>Alto</v>
       </c>
       <c r="G105">
@@ -4226,7 +4160,7 @@
         <v>19</v>
       </c>
       <c r="F106" t="str">
-        <f>IF(Dati_grezzi!C106&lt;=$O$2,"Basso",IF(C106&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C106&lt;=$J$2,"Basso",IF(C106&lt;=$J$3,"Medio","Alto"))</f>
         <v>Alto</v>
       </c>
       <c r="G106">
@@ -4250,7 +4184,7 @@
         <v>19</v>
       </c>
       <c r="F107" t="str">
-        <f>IF(Dati_grezzi!C107&lt;=$O$2,"Basso",IF(C107&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C107&lt;=$J$2,"Basso",IF(C107&lt;=$J$3,"Medio","Alto"))</f>
         <v>Alto</v>
       </c>
       <c r="G107">
@@ -4274,7 +4208,7 @@
         <v>19</v>
       </c>
       <c r="F108" t="str">
-        <f>IF(Dati_grezzi!C108&lt;=$O$2,"Basso",IF(C108&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C108&lt;=$J$2,"Basso",IF(C108&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G108">
@@ -4298,7 +4232,7 @@
         <v>19</v>
       </c>
       <c r="F109" t="str">
-        <f>IF(Dati_grezzi!C109&lt;=$O$2,"Basso",IF(C109&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C109&lt;=$J$2,"Basso",IF(C109&lt;=$J$3,"Medio","Alto"))</f>
         <v>Alto</v>
       </c>
       <c r="G109">
@@ -4322,7 +4256,7 @@
         <v>19</v>
       </c>
       <c r="F110" t="str">
-        <f>IF(Dati_grezzi!C110&lt;=$O$2,"Basso",IF(C110&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C110&lt;=$J$2,"Basso",IF(C110&lt;=$J$3,"Medio","Alto"))</f>
         <v>Alto</v>
       </c>
       <c r="G110">
@@ -4346,7 +4280,7 @@
         <v>19</v>
       </c>
       <c r="F111" t="str">
-        <f>IF(Dati_grezzi!C111&lt;=$O$2,"Basso",IF(C111&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C111&lt;=$J$2,"Basso",IF(C111&lt;=$J$3,"Medio","Alto"))</f>
         <v>Alto</v>
       </c>
       <c r="G111">
@@ -4370,7 +4304,7 @@
         <v>19</v>
       </c>
       <c r="F112" t="str">
-        <f>IF(Dati_grezzi!C112&lt;=$O$2,"Basso",IF(C112&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C112&lt;=$J$2,"Basso",IF(C112&lt;=$J$3,"Medio","Alto"))</f>
         <v>Alto</v>
       </c>
       <c r="G112">
@@ -4394,7 +4328,7 @@
         <v>19</v>
       </c>
       <c r="F113" t="str">
-        <f>IF(Dati_grezzi!C113&lt;=$O$2,"Basso",IF(C113&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C113&lt;=$J$2,"Basso",IF(C113&lt;=$J$3,"Medio","Alto"))</f>
         <v>Alto</v>
       </c>
       <c r="G113">
@@ -4418,7 +4352,7 @@
         <v>19</v>
       </c>
       <c r="F114" t="str">
-        <f>IF(Dati_grezzi!C114&lt;=$O$2,"Basso",IF(C114&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C114&lt;=$J$2,"Basso",IF(C114&lt;=$J$3,"Medio","Alto"))</f>
         <v>Alto</v>
       </c>
       <c r="G114">
@@ -4442,7 +4376,7 @@
         <v>19</v>
       </c>
       <c r="F115" t="str">
-        <f>IF(Dati_grezzi!C115&lt;=$O$2,"Basso",IF(C115&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C115&lt;=$J$2,"Basso",IF(C115&lt;=$J$3,"Medio","Alto"))</f>
         <v>Alto</v>
       </c>
       <c r="G115">
@@ -4466,7 +4400,7 @@
         <v>19</v>
       </c>
       <c r="F116" t="str">
-        <f>IF(Dati_grezzi!C116&lt;=$O$2,"Basso",IF(C116&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C116&lt;=$J$2,"Basso",IF(C116&lt;=$J$3,"Medio","Alto"))</f>
         <v>Alto</v>
       </c>
       <c r="G116">
@@ -4490,7 +4424,7 @@
         <v>19</v>
       </c>
       <c r="F117" t="str">
-        <f>IF(Dati_grezzi!C117&lt;=$O$2,"Basso",IF(C117&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C117&lt;=$J$2,"Basso",IF(C117&lt;=$J$3,"Medio","Alto"))</f>
         <v>Alto</v>
       </c>
       <c r="G117">
@@ -4514,7 +4448,7 @@
         <v>19</v>
       </c>
       <c r="F118" t="str">
-        <f>IF(Dati_grezzi!C118&lt;=$O$2,"Basso",IF(C118&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C118&lt;=$J$2,"Basso",IF(C118&lt;=$J$3,"Medio","Alto"))</f>
         <v>Alto</v>
       </c>
       <c r="G118">
@@ -4538,7 +4472,7 @@
         <v>19</v>
       </c>
       <c r="F119" t="str">
-        <f>IF(Dati_grezzi!C119&lt;=$O$2,"Basso",IF(C119&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C119&lt;=$J$2,"Basso",IF(C119&lt;=$J$3,"Medio","Alto"))</f>
         <v>Alto</v>
       </c>
       <c r="G119">
@@ -4562,7 +4496,7 @@
         <v>19</v>
       </c>
       <c r="F120" t="str">
-        <f>IF(Dati_grezzi!C120&lt;=$O$2,"Basso",IF(C120&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C120&lt;=$J$2,"Basso",IF(C120&lt;=$J$3,"Medio","Alto"))</f>
         <v>Alto</v>
       </c>
       <c r="G120">
@@ -4586,7 +4520,7 @@
         <v>19</v>
       </c>
       <c r="F121" t="str">
-        <f>IF(Dati_grezzi!C121&lt;=$O$2,"Basso",IF(C121&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C121&lt;=$J$2,"Basso",IF(C121&lt;=$J$3,"Medio","Alto"))</f>
         <v>Alto</v>
       </c>
       <c r="G121">
@@ -4610,7 +4544,7 @@
         <v>19</v>
       </c>
       <c r="F122" t="str">
-        <f>IF(Dati_grezzi!C122&lt;=$O$2,"Basso",IF(C122&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C122&lt;=$J$2,"Basso",IF(C122&lt;=$J$3,"Medio","Alto"))</f>
         <v>Alto</v>
       </c>
       <c r="G122">
@@ -4634,7 +4568,7 @@
         <v>19</v>
       </c>
       <c r="F123" t="str">
-        <f>IF(Dati_grezzi!C123&lt;=$O$2,"Basso",IF(C123&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C123&lt;=$J$2,"Basso",IF(C123&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G123">
@@ -4658,7 +4592,7 @@
         <v>19</v>
       </c>
       <c r="F124" t="str">
-        <f>IF(Dati_grezzi!C124&lt;=$O$2,"Basso",IF(C124&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C124&lt;=$J$2,"Basso",IF(C124&lt;=$J$3,"Medio","Alto"))</f>
         <v>Alto</v>
       </c>
       <c r="G124">
@@ -4682,7 +4616,7 @@
         <v>19</v>
       </c>
       <c r="F125" t="str">
-        <f>IF(Dati_grezzi!C125&lt;=$O$2,"Basso",IF(C125&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C125&lt;=$J$2,"Basso",IF(C125&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G125">
@@ -4706,7 +4640,7 @@
         <v>19</v>
       </c>
       <c r="F126" t="str">
-        <f>IF(Dati_grezzi!C126&lt;=$O$2,"Basso",IF(C126&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C126&lt;=$J$2,"Basso",IF(C126&lt;=$J$3,"Medio","Alto"))</f>
         <v>Alto</v>
       </c>
       <c r="G126">
@@ -4730,7 +4664,7 @@
         <v>19</v>
       </c>
       <c r="F127" t="str">
-        <f>IF(Dati_grezzi!C127&lt;=$O$2,"Basso",IF(C127&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C127&lt;=$J$2,"Basso",IF(C127&lt;=$J$3,"Medio","Alto"))</f>
         <v>Alto</v>
       </c>
       <c r="G127">
@@ -4754,7 +4688,7 @@
         <v>19</v>
       </c>
       <c r="F128" t="str">
-        <f>IF(Dati_grezzi!C128&lt;=$O$2,"Basso",IF(C128&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C128&lt;=$J$2,"Basso",IF(C128&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G128">
@@ -4778,7 +4712,7 @@
         <v>19</v>
       </c>
       <c r="F129" t="str">
-        <f>IF(Dati_grezzi!C129&lt;=$O$2,"Basso",IF(C129&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C129&lt;=$J$2,"Basso",IF(C129&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G129">
@@ -4802,7 +4736,7 @@
         <v>19</v>
       </c>
       <c r="F130" t="str">
-        <f>IF(Dati_grezzi!C130&lt;=$O$2,"Basso",IF(C130&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C130&lt;=$J$2,"Basso",IF(C130&lt;=$J$3,"Medio","Alto"))</f>
         <v>Alto</v>
       </c>
       <c r="G130">
@@ -4826,7 +4760,7 @@
         <v>19</v>
       </c>
       <c r="F131" t="str">
-        <f>IF(Dati_grezzi!C131&lt;=$O$2,"Basso",IF(C131&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C131&lt;=$J$2,"Basso",IF(C131&lt;=$J$3,"Medio","Alto"))</f>
         <v>Alto</v>
       </c>
       <c r="G131">
@@ -4850,7 +4784,7 @@
         <v>19</v>
       </c>
       <c r="F132" t="str">
-        <f>IF(Dati_grezzi!C132&lt;=$O$2,"Basso",IF(C132&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C132&lt;=$J$2,"Basso",IF(C132&lt;=$J$3,"Medio","Alto"))</f>
         <v>Alto</v>
       </c>
       <c r="G132">
@@ -4874,7 +4808,7 @@
         <v>19</v>
       </c>
       <c r="F133" t="str">
-        <f>IF(Dati_grezzi!C133&lt;=$O$2,"Basso",IF(C133&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C133&lt;=$J$2,"Basso",IF(C133&lt;=$J$3,"Medio","Alto"))</f>
         <v>Alto</v>
       </c>
       <c r="G133">
@@ -4898,7 +4832,7 @@
         <v>19</v>
       </c>
       <c r="F134" t="str">
-        <f>IF(Dati_grezzi!C134&lt;=$O$2,"Basso",IF(C134&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C134&lt;=$J$2,"Basso",IF(C134&lt;=$J$3,"Medio","Alto"))</f>
         <v>Alto</v>
       </c>
       <c r="G134">
@@ -4922,7 +4856,7 @@
         <v>19</v>
       </c>
       <c r="F135" t="str">
-        <f>IF(Dati_grezzi!C135&lt;=$O$2,"Basso",IF(C135&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C135&lt;=$J$2,"Basso",IF(C135&lt;=$J$3,"Medio","Alto"))</f>
         <v>Alto</v>
       </c>
       <c r="G135">
@@ -4946,7 +4880,7 @@
         <v>19</v>
       </c>
       <c r="F136" t="str">
-        <f>IF(Dati_grezzi!C136&lt;=$O$2,"Basso",IF(C136&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C136&lt;=$J$2,"Basso",IF(C136&lt;=$J$3,"Medio","Alto"))</f>
         <v>Alto</v>
       </c>
       <c r="G136">
@@ -4970,7 +4904,7 @@
         <v>19</v>
       </c>
       <c r="F137" t="str">
-        <f>IF(Dati_grezzi!C137&lt;=$O$2,"Basso",IF(C137&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C137&lt;=$J$2,"Basso",IF(C137&lt;=$J$3,"Medio","Alto"))</f>
         <v>Alto</v>
       </c>
       <c r="G137">
@@ -4994,7 +4928,7 @@
         <v>19</v>
       </c>
       <c r="F138" t="str">
-        <f>IF(Dati_grezzi!C138&lt;=$O$2,"Basso",IF(C138&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C138&lt;=$J$2,"Basso",IF(C138&lt;=$J$3,"Medio","Alto"))</f>
         <v>Alto</v>
       </c>
       <c r="G138">
@@ -5018,7 +4952,7 @@
         <v>19</v>
       </c>
       <c r="F139" t="str">
-        <f>IF(Dati_grezzi!C139&lt;=$O$2,"Basso",IF(C139&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C139&lt;=$J$2,"Basso",IF(C139&lt;=$J$3,"Medio","Alto"))</f>
         <v>Alto</v>
       </c>
       <c r="G139">
@@ -5042,7 +4976,7 @@
         <v>19</v>
       </c>
       <c r="F140" t="str">
-        <f>IF(Dati_grezzi!C140&lt;=$O$2,"Basso",IF(C140&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C140&lt;=$J$2,"Basso",IF(C140&lt;=$J$3,"Medio","Alto"))</f>
         <v>Medio</v>
       </c>
       <c r="G140">
@@ -5066,7 +5000,7 @@
         <v>19</v>
       </c>
       <c r="F141" t="str">
-        <f>IF(Dati_grezzi!C141&lt;=$O$2,"Basso",IF(C141&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C141&lt;=$J$2,"Basso",IF(C141&lt;=$J$3,"Medio","Alto"))</f>
         <v>Alto</v>
       </c>
       <c r="G141">
@@ -5090,7 +5024,7 @@
         <v>19</v>
       </c>
       <c r="F142" t="str">
-        <f>IF(Dati_grezzi!C142&lt;=$O$2,"Basso",IF(C142&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C142&lt;=$J$2,"Basso",IF(C142&lt;=$J$3,"Medio","Alto"))</f>
         <v>Alto</v>
       </c>
       <c r="G142">
@@ -5114,7 +5048,7 @@
         <v>19</v>
       </c>
       <c r="F143" t="str">
-        <f>IF(Dati_grezzi!C143&lt;=$O$2,"Basso",IF(C143&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C143&lt;=$J$2,"Basso",IF(C143&lt;=$J$3,"Medio","Alto"))</f>
         <v>Alto</v>
       </c>
       <c r="G143">
@@ -5138,7 +5072,7 @@
         <v>19</v>
       </c>
       <c r="F144" t="str">
-        <f>IF(Dati_grezzi!C144&lt;=$O$2,"Basso",IF(C144&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C144&lt;=$J$2,"Basso",IF(C144&lt;=$J$3,"Medio","Alto"))</f>
         <v>Alto</v>
       </c>
       <c r="G144">
@@ -5162,7 +5096,7 @@
         <v>19</v>
       </c>
       <c r="F145" t="str">
-        <f>IF(Dati_grezzi!C145&lt;=$O$2,"Basso",IF(C145&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C145&lt;=$J$2,"Basso",IF(C145&lt;=$J$3,"Medio","Alto"))</f>
         <v>Alto</v>
       </c>
       <c r="G145">
@@ -5186,7 +5120,7 @@
         <v>19</v>
       </c>
       <c r="F146" t="str">
-        <f>IF(Dati_grezzi!C146&lt;=$O$2,"Basso",IF(C146&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C146&lt;=$J$2,"Basso",IF(C146&lt;=$J$3,"Medio","Alto"))</f>
         <v>Alto</v>
       </c>
       <c r="G146">
@@ -5210,7 +5144,7 @@
         <v>19</v>
       </c>
       <c r="F147" t="str">
-        <f>IF(Dati_grezzi!C147&lt;=$O$2,"Basso",IF(C147&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C147&lt;=$J$2,"Basso",IF(C147&lt;=$J$3,"Medio","Alto"))</f>
         <v>Alto</v>
       </c>
       <c r="G147">
@@ -5234,7 +5168,7 @@
         <v>19</v>
       </c>
       <c r="F148" t="str">
-        <f>IF(Dati_grezzi!C148&lt;=$O$2,"Basso",IF(C148&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C148&lt;=$J$2,"Basso",IF(C148&lt;=$J$3,"Medio","Alto"))</f>
         <v>Alto</v>
       </c>
       <c r="G148">
@@ -5258,7 +5192,7 @@
         <v>19</v>
       </c>
       <c r="F149" t="str">
-        <f>IF(Dati_grezzi!C149&lt;=$O$2,"Basso",IF(C149&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C149&lt;=$J$2,"Basso",IF(C149&lt;=$J$3,"Medio","Alto"))</f>
         <v>Alto</v>
       </c>
       <c r="G149">
@@ -5282,7 +5216,7 @@
         <v>19</v>
       </c>
       <c r="F150" t="str">
-        <f>IF(Dati_grezzi!C150&lt;=$O$2,"Basso",IF(C150&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C150&lt;=$J$2,"Basso",IF(C150&lt;=$J$3,"Medio","Alto"))</f>
         <v>Alto</v>
       </c>
       <c r="G150">
@@ -5306,7 +5240,7 @@
         <v>19</v>
       </c>
       <c r="F151" t="str">
-        <f>IF(Dati_grezzi!C151&lt;=$O$2,"Basso",IF(C151&lt;=$O$3,"Medio","Alto"))</f>
+        <f>IF(Dati_grezzi!C151&lt;=$J$2,"Basso",IF(C151&lt;=$J$3,"Medio","Alto"))</f>
         <v>Alto</v>
       </c>
       <c r="G151">
@@ -10648,556 +10582,6 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E32CF21-0BFF-4609-807B-E20BDED60E91}">
-  <dimension ref="A1:C50"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="9.7109375" customWidth="1"/>
-    <col min="3" max="3" width="12" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>19</v>
-      </c>
-      <c r="B4" t="s">
-        <v>56</v>
-      </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>19</v>
-      </c>
-      <c r="B5" t="s">
-        <v>56</v>
-      </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>19</v>
-      </c>
-      <c r="B6" t="s">
-        <v>56</v>
-      </c>
-      <c r="C6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>19</v>
-      </c>
-      <c r="B7" t="s">
-        <v>56</v>
-      </c>
-      <c r="C7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>19</v>
-      </c>
-      <c r="B8" t="s">
-        <v>56</v>
-      </c>
-      <c r="C8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>19</v>
-      </c>
-      <c r="B9" t="s">
-        <v>56</v>
-      </c>
-      <c r="C9">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>19</v>
-      </c>
-      <c r="B10" t="s">
-        <v>56</v>
-      </c>
-      <c r="C10">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>19</v>
-      </c>
-      <c r="B11" t="s">
-        <v>56</v>
-      </c>
-      <c r="C11">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>19</v>
-      </c>
-      <c r="B12" t="s">
-        <v>56</v>
-      </c>
-      <c r="C12">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>19</v>
-      </c>
-      <c r="B13" t="s">
-        <v>56</v>
-      </c>
-      <c r="C13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>19</v>
-      </c>
-      <c r="B14" t="s">
-        <v>56</v>
-      </c>
-      <c r="C14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>19</v>
-      </c>
-      <c r="B15" t="s">
-        <v>56</v>
-      </c>
-      <c r="C15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>19</v>
-      </c>
-      <c r="B16" t="s">
-        <v>56</v>
-      </c>
-      <c r="C16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>19</v>
-      </c>
-      <c r="B17" t="s">
-        <v>56</v>
-      </c>
-      <c r="C17">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>19</v>
-      </c>
-      <c r="B18" t="s">
-        <v>56</v>
-      </c>
-      <c r="C18">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>19</v>
-      </c>
-      <c r="B19" t="s">
-        <v>56</v>
-      </c>
-      <c r="C19">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>19</v>
-      </c>
-      <c r="B20" t="s">
-        <v>56</v>
-      </c>
-      <c r="C20">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>19</v>
-      </c>
-      <c r="B21" t="s">
-        <v>56</v>
-      </c>
-      <c r="C21">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>19</v>
-      </c>
-      <c r="B22" t="s">
-        <v>56</v>
-      </c>
-      <c r="C22">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>19</v>
-      </c>
-      <c r="B23" t="s">
-        <v>56</v>
-      </c>
-      <c r="C23">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>19</v>
-      </c>
-      <c r="B24" t="s">
-        <v>56</v>
-      </c>
-      <c r="C24">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>19</v>
-      </c>
-      <c r="B25" t="s">
-        <v>56</v>
-      </c>
-      <c r="C25">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>19</v>
-      </c>
-      <c r="B26" t="s">
-        <v>56</v>
-      </c>
-      <c r="C26">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>19</v>
-      </c>
-      <c r="B27" t="s">
-        <v>56</v>
-      </c>
-      <c r="C27">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>19</v>
-      </c>
-      <c r="B28" t="s">
-        <v>56</v>
-      </c>
-      <c r="C28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>19</v>
-      </c>
-      <c r="B29" t="s">
-        <v>56</v>
-      </c>
-      <c r="C29">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>19</v>
-      </c>
-      <c r="B30" t="s">
-        <v>56</v>
-      </c>
-      <c r="C30">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>19</v>
-      </c>
-      <c r="B31" t="s">
-        <v>56</v>
-      </c>
-      <c r="C31">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>19</v>
-      </c>
-      <c r="B32" t="s">
-        <v>56</v>
-      </c>
-      <c r="C32">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>19</v>
-      </c>
-      <c r="B33" t="s">
-        <v>56</v>
-      </c>
-      <c r="C33">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>19</v>
-      </c>
-      <c r="B34" t="s">
-        <v>56</v>
-      </c>
-      <c r="C34">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>19</v>
-      </c>
-      <c r="B35" t="s">
-        <v>56</v>
-      </c>
-      <c r="C35">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>19</v>
-      </c>
-      <c r="B36" t="s">
-        <v>56</v>
-      </c>
-      <c r="C36">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>19</v>
-      </c>
-      <c r="B37" t="s">
-        <v>56</v>
-      </c>
-      <c r="C37">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>19</v>
-      </c>
-      <c r="B38" t="s">
-        <v>56</v>
-      </c>
-      <c r="C38">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>19</v>
-      </c>
-      <c r="B39" t="s">
-        <v>56</v>
-      </c>
-      <c r="C39">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>19</v>
-      </c>
-      <c r="B40" t="s">
-        <v>56</v>
-      </c>
-      <c r="C40">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
-        <v>19</v>
-      </c>
-      <c r="B41" t="s">
-        <v>56</v>
-      </c>
-      <c r="C41">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
-        <v>19</v>
-      </c>
-      <c r="B42" t="s">
-        <v>56</v>
-      </c>
-      <c r="C42">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
-        <v>19</v>
-      </c>
-      <c r="B43" t="s">
-        <v>56</v>
-      </c>
-      <c r="C43">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
-        <v>19</v>
-      </c>
-      <c r="B44" t="s">
-        <v>56</v>
-      </c>
-      <c r="C44">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
-        <v>19</v>
-      </c>
-      <c r="B45" t="s">
-        <v>56</v>
-      </c>
-      <c r="C45">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
-        <v>19</v>
-      </c>
-      <c r="B46" t="s">
-        <v>56</v>
-      </c>
-      <c r="C46">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
-        <v>19</v>
-      </c>
-      <c r="B47" t="s">
-        <v>56</v>
-      </c>
-      <c r="C47">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
-        <v>19</v>
-      </c>
-      <c r="B48" t="s">
-        <v>56</v>
-      </c>
-      <c r="C48">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
-        <v>19</v>
-      </c>
-      <c r="B49" t="s">
-        <v>56</v>
-      </c>
-      <c r="C49">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
-        <v>19</v>
-      </c>
-      <c r="B50" t="s">
-        <v>56</v>
-      </c>
-      <c r="C50">
-        <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96728C41-8E02-447C-B88F-59C6DBB20D94}">
   <dimension ref="A2:E22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -11243,12 +10627,10 @@
       <c r="A5" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="B5" s="13"/>
-      <c r="C5" s="13">
+      <c r="C5">
         <v>50</v>
       </c>
-      <c r="D5" s="13"/>
-      <c r="E5" s="13">
+      <c r="E5">
         <v>50</v>
       </c>
     </row>
@@ -11256,14 +10638,13 @@
       <c r="A6" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="13">
+      <c r="B6">
         <v>2</v>
       </c>
-      <c r="C6" s="13"/>
-      <c r="D6" s="13">
+      <c r="D6">
         <v>48</v>
       </c>
-      <c r="E6" s="13">
+      <c r="E6">
         <v>50</v>
       </c>
     </row>
@@ -11271,14 +10652,13 @@
       <c r="A7" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="13">
+      <c r="B7">
         <v>44</v>
       </c>
-      <c r="C7" s="13"/>
-      <c r="D7" s="13">
+      <c r="D7">
         <v>6</v>
       </c>
-      <c r="E7" s="13">
+      <c r="E7">
         <v>50</v>
       </c>
     </row>
@@ -11286,16 +10666,16 @@
       <c r="A8" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="B8" s="13">
+      <c r="B8">
         <v>46</v>
       </c>
-      <c r="C8" s="13">
+      <c r="C8">
         <v>50</v>
       </c>
-      <c r="D8" s="13">
+      <c r="D8">
         <v>54</v>
       </c>
-      <c r="E8" s="13">
+      <c r="E8">
         <v>150</v>
       </c>
     </row>
@@ -11383,14 +10763,61 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+  <dimension ref="A1:A9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="120" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>69</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="674b27b8-e1cd-4723-9694-0b904cc35f92">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -11572,20 +10999,19 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="674b27b8-e1cd-4723-9694-0b904cc35f92">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A9910A44-9D4B-4AE0-8F32-468CD0F680ED}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CBAACB6A-3780-4878-A77A-6EE417743D34}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="674b27b8-e1cd-4723-9694-0b904cc35f92"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -11609,9 +11035,11 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CBAACB6A-3780-4878-A77A-6EE417743D34}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A9910A44-9D4B-4AE0-8F32-468CD0F680ED}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="674b27b8-e1cd-4723-9694-0b904cc35f92"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>